<commit_message>
sorry - forgot to include LinCuboid into tests main
</commit_message>
<xml_diff>
--- a/Matthai_UnitTesting2018.xlsx
+++ b/Matthai_UnitTesting2018.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="28028"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <bookViews>
-    <workbookView xWindow="21960" yWindow="9420" windowWidth="28960" windowHeight="20560" tabRatio="500"/>
+    <workbookView xWindow="5740" yWindow="8840" windowWidth="28960" windowHeight="20560" tabRatio="500" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Existing Tests - Not Running" sheetId="1" r:id="rId1"/>
@@ -21,10 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
-  <si>
-    <t>Missin</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="13">
   <si>
     <t>Unit Tests that exist, but are not being run (August 2018)</t>
   </si>
@@ -42,13 +39,34 @@
   </si>
   <si>
     <t>Boundary_Test</t>
+  </si>
+  <si>
+    <t>yes</t>
+  </si>
+  <si>
+    <t>Actions</t>
+  </si>
+  <si>
+    <t>automatically test interpolation function derivative matrix</t>
+  </si>
+  <si>
+    <t>Unit Tests that are missing (August 2018)</t>
+  </si>
+  <si>
+    <t>LinearRectangle_Test</t>
+  </si>
+  <si>
+    <t>Originator (class/test)</t>
+  </si>
+  <si>
+    <t>Hani</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -60,6 +78,22 @@
       <b/>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="12"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="12"/>
+      <color theme="11"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -82,14 +116,18 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="3">
+    <cellStyle name="Followed Hyperlink" xfId="2" builtinId="9" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8" hidden="1"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -419,40 +457,50 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0"/>
   <cols>
     <col min="1" max="1" width="22.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="1" customFormat="1">
+    <row r="1" spans="1:4" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:3">
-      <c r="A3" t="s">
+      <c r="B3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C3" t="s">
         <v>2</v>
       </c>
-      <c r="B3" t="s">
+      <c r="D3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4">
+      <c r="A11" t="s">
         <v>4</v>
       </c>
-      <c r="C3" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3">
-      <c r="A4" t="s">
+      <c r="B11" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="11" spans="1:3">
-      <c r="A11" t="s">
-        <v>5</v>
+      <c r="D11" t="s">
+        <v>8</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967292" verticalDpi="4294967292"/>
   <extLst>
     <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{64002731-A6B0-56B0-2670-7721B7C09600}">
       <mx:PLV Mode="0" OnePage="0" WScale="0"/>
@@ -463,12 +511,43 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0"/>
+  <cols>
+    <col min="1" max="1" width="28.33203125" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:1">
-      <c r="A1" t="s">
-        <v>0</v>
+    <row r="1" spans="1:5">
+      <c r="A1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D3" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E4" t="s">
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: tracking unit tests that are not being run
</commit_message>
<xml_diff>
--- a/Matthai_UnitTesting2018.xlsx
+++ b/Matthai_UnitTesting2018.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="28028"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <bookViews>
-    <workbookView xWindow="5740" yWindow="8840" windowWidth="28960" windowHeight="20560" tabRatio="500" activeTab="1"/>
+    <workbookView xWindow="1140" yWindow="8860" windowWidth="28960" windowHeight="20560" tabRatio="500"/>
   </bookViews>
   <sheets>
     <sheet name="Existing Tests - Not Running" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="47">
   <si>
     <t>Unit Tests that exist, but are not being run (August 2018)</t>
   </si>
@@ -60,16 +60,125 @@
   </si>
   <si>
     <t>Hani</t>
+  </si>
+  <si>
+    <t>ConstraintPointToNodePropertyVisitor_Test</t>
+  </si>
+  <si>
+    <t>refactor</t>
+  </si>
+  <si>
+    <t>CopyReplaceVisitor_Test</t>
+  </si>
+  <si>
+    <t>CsmpIntro1_TestCase</t>
+  </si>
+  <si>
+    <t>ElementPolicyIntegrity_Test</t>
+  </si>
+  <si>
+    <t>tests stand-alone element</t>
+  </si>
+  <si>
+    <t>FiniteVolumeTransportBasics_Test</t>
+  </si>
+  <si>
+    <t>FluxMIsmatch</t>
+  </si>
+  <si>
+    <t>GenericFiniteVolumeTransport_Test</t>
+  </si>
+  <si>
+    <t>geometricCalculations_Test</t>
+  </si>
+  <si>
+    <t>length and dotproduct</t>
+  </si>
+  <si>
+    <t>needs to test all other enlisted functionality</t>
+  </si>
+  <si>
+    <t>Integral_var_NT_lhsop_N_dV_Test</t>
+  </si>
+  <si>
+    <t>Integral_var_NT_rhsop_N_dV_Test</t>
+  </si>
+  <si>
+    <t>compiles</t>
+  </si>
+  <si>
+    <t>incomplete</t>
+  </si>
+  <si>
+    <t>Mesh_Test</t>
+  </si>
+  <si>
+    <t>refactor for MeshManager (memory allocation etc.)</t>
+  </si>
+  <si>
+    <t>ModelSubdomain_Test</t>
+  </si>
+  <si>
+    <t>running</t>
+  </si>
+  <si>
+    <t>add key functionality tests</t>
+  </si>
+  <si>
+    <t>Parallel_TestCase</t>
+  </si>
+  <si>
+    <t>InterFace</t>
+  </si>
+  <si>
+    <t>PDE_Integrator_CRM</t>
+  </si>
+  <si>
+    <t>Placement_Test</t>
+  </si>
+  <si>
+    <t>add better cases so the results really show if there are problems</t>
+  </si>
+  <si>
+    <t>PropertyStorageSpeed_Test</t>
+  </si>
+  <si>
+    <t>for profiling</t>
+  </si>
+  <si>
+    <t>run</t>
+  </si>
+  <si>
+    <t>RelativePermeabilityModel_Test</t>
+  </si>
+  <si>
+    <t>StatisticalAnalyzer_Test</t>
+  </si>
+  <si>
+    <t>Variables_Test</t>
+  </si>
+  <si>
+    <t>Author</t>
+  </si>
+  <si>
+    <t>P. Lang</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -118,11 +227,12 @@
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
@@ -457,44 +567,195 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0"/>
   <cols>
-    <col min="1" max="1" width="22.1640625" customWidth="1"/>
+    <col min="1" max="1" width="39.83203125" customWidth="1"/>
+    <col min="2" max="2" width="25.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="1" customFormat="1">
+    <row r="1" spans="1:5" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4">
-      <c r="A3" t="s">
+    <row r="3" spans="1:5">
+      <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E3" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:4">
+    <row r="4" spans="1:5">
       <c r="A4" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:4">
-      <c r="A11" t="s">
+    <row r="5" spans="1:5">
+      <c r="A5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
+      <c r="A7" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5">
+      <c r="A8" t="s">
+        <v>17</v>
+      </c>
+      <c r="B8" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5">
+      <c r="A9" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5">
+      <c r="A10" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5">
+      <c r="A11" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5">
+      <c r="A12" t="s">
+        <v>22</v>
+      </c>
+      <c r="B12" t="s">
+        <v>23</v>
+      </c>
+      <c r="C12" t="s">
+        <v>28</v>
+      </c>
+      <c r="E12" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5">
+      <c r="A13" t="s">
+        <v>25</v>
+      </c>
+      <c r="C13" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5">
+      <c r="A14" t="s">
+        <v>26</v>
+      </c>
+      <c r="C14" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5">
+      <c r="A15" t="s">
+        <v>29</v>
+      </c>
+      <c r="C15" t="s">
+        <v>28</v>
+      </c>
+      <c r="E15" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5">
+      <c r="A16" t="s">
+        <v>31</v>
+      </c>
+      <c r="B16" t="s">
+        <v>32</v>
+      </c>
+      <c r="C16" t="s">
+        <v>28</v>
+      </c>
+      <c r="E16" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5">
+      <c r="A17" t="s">
+        <v>34</v>
+      </c>
+      <c r="C17" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5">
+      <c r="A18" t="s">
+        <v>37</v>
+      </c>
+      <c r="C18" t="s">
+        <v>27</v>
+      </c>
+      <c r="E18" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5">
+      <c r="A19" t="s">
+        <v>39</v>
+      </c>
+      <c r="B19" t="s">
+        <v>40</v>
+      </c>
+      <c r="C19" t="s">
+        <v>27</v>
+      </c>
+      <c r="E19" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5">
+      <c r="A20" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5">
+      <c r="A21" s="2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5">
+      <c r="A22" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="D22" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4">
+      <c r="A34" t="s">
         <v>4</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B34" t="s">
         <v>6</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D34" t="s">
         <v>8</v>
       </c>
     </row>
@@ -511,7 +772,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0"/>
   <cols>
     <col min="1" max="1" width="28.33203125" customWidth="1"/>
@@ -547,6 +808,19 @@
         <v>10</v>
       </c>
       <c r="E4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="A5" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6" t="s">
+        <v>36</v>
+      </c>
+      <c r="E6" t="s">
         <v>12</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: got P. Lang's Variables_Test running again; it still needs to be refactored so that it contains a SplitBoundary so that InterFace variable read/write is tested
</commit_message>
<xml_diff>
--- a/Matthai_UnitTesting2018.xlsx
+++ b/Matthai_UnitTesting2018.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="48">
   <si>
     <t>Unit Tests that exist, but are not being run (August 2018)</t>
   </si>
@@ -162,6 +162,9 @@
   </si>
   <si>
     <t>P. Lang</t>
+  </si>
+  <si>
+    <t>needs to include SplitBoundary object</t>
   </si>
 </sst>
 </file>
@@ -744,8 +747,14 @@
       <c r="A22" s="2" t="s">
         <v>44</v>
       </c>
+      <c r="B22" t="s">
+        <v>47</v>
+      </c>
       <c r="D22" t="s">
         <v>46</v>
+      </c>
+      <c r="E22" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="34" spans="1:4">

</xml_diff>